<commit_message>
feat: Integrate Meals Waste and Vegetable Waste questions into Canteen Waste logs
</commit_message>
<xml_diff>
--- a/canteen_waste_log.xlsx
+++ b/canteen_waste_log.xlsx
@@ -723,7 +723,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="32" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -791,6 +791,10 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="24" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1246,7 +1250,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:D35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="2" max="2"/>
@@ -1258,7 +1262,9 @@
           <t xml:space="preserve">               BARANI HYDRAULICS INDIA PRIVATE LIMITED</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="23" t="n"/>
+      <c r="C1" s="24" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DOC NO: R/MAI/CW
 MONTH/YEAR: </t>
@@ -1272,6 +1278,8 @@
           <t>CANTEEN WASTE LOG</t>
         </is>
       </c>
+      <c r="C2" s="25" t="n"/>
+      <c r="D2" s="26" t="n"/>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
@@ -1281,6 +1289,16 @@
       </c>
       <c r="B3" s="10" t="inlineStr">
         <is>
+          <t>MEALS WASTE (KG)</t>
+        </is>
+      </c>
+      <c r="C3" s="10" t="inlineStr">
+        <is>
+          <t>VEGETABLE WASTE (KG)</t>
+        </is>
+      </c>
+      <c r="D3" s="10" t="inlineStr">
+        <is>
           <t>CARETAKER SIGN</t>
         </is>
       </c>
@@ -1290,90 +1308,120 @@
         <v>1</v>
       </c>
       <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
     </row>
     <row r="5" ht="33" customHeight="1">
       <c r="A5" s="12" t="n">
         <v>2</v>
       </c>
       <c r="B5" s="13" t="n"/>
+      <c r="C5" s="13" t="n"/>
+      <c r="D5" s="13" t="n"/>
     </row>
     <row r="6" ht="33" customHeight="1">
       <c r="A6" s="12" t="n">
         <v>3</v>
       </c>
       <c r="B6" s="13" t="n"/>
+      <c r="C6" s="13" t="n"/>
+      <c r="D6" s="13" t="n"/>
     </row>
     <row r="7" ht="33" customHeight="1">
       <c r="A7" s="12" t="n">
         <v>4</v>
       </c>
       <c r="B7" s="13" t="n"/>
+      <c r="C7" s="13" t="n"/>
+      <c r="D7" s="13" t="n"/>
     </row>
     <row r="8" ht="33" customHeight="1">
       <c r="A8" s="12" t="n">
         <v>5</v>
       </c>
       <c r="B8" s="13" t="n"/>
+      <c r="C8" s="13" t="n"/>
+      <c r="D8" s="13" t="n"/>
     </row>
     <row r="9" ht="33" customHeight="1">
       <c r="A9" s="12" t="n">
         <v>6</v>
       </c>
       <c r="B9" s="13" t="n"/>
+      <c r="C9" s="13" t="n"/>
+      <c r="D9" s="13" t="n"/>
     </row>
     <row r="10" ht="33" customHeight="1">
       <c r="A10" s="15" t="n">
         <v>7</v>
       </c>
       <c r="B10" s="16" t="n"/>
+      <c r="C10" s="16" t="n"/>
+      <c r="D10" s="16" t="n"/>
     </row>
     <row r="11" ht="33" customHeight="1">
       <c r="A11" s="12" t="n">
         <v>8</v>
       </c>
       <c r="B11" s="13" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="D11" s="13" t="n"/>
     </row>
     <row r="12" ht="33" customHeight="1">
       <c r="A12" s="12" t="n">
         <v>9</v>
       </c>
       <c r="B12" s="13" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="D12" s="13" t="n"/>
     </row>
     <row r="13" ht="33" customHeight="1">
       <c r="A13" s="12" t="n">
         <v>10</v>
       </c>
       <c r="B13" s="13" t="n"/>
+      <c r="C13" s="13" t="n"/>
+      <c r="D13" s="13" t="n"/>
     </row>
     <row r="14" ht="33" customHeight="1">
       <c r="A14" s="12" t="n">
         <v>11</v>
       </c>
       <c r="B14" s="13" t="n"/>
+      <c r="C14" s="13" t="n"/>
+      <c r="D14" s="13" t="n"/>
     </row>
     <row r="15" ht="33" customHeight="1">
       <c r="A15" s="12" t="n">
         <v>12</v>
       </c>
       <c r="B15" s="13" t="n"/>
+      <c r="C15" s="13" t="n"/>
+      <c r="D15" s="13" t="n"/>
     </row>
     <row r="16" ht="33" customHeight="1">
       <c r="A16" s="12" t="n">
         <v>13</v>
       </c>
       <c r="B16" s="13" t="n"/>
+      <c r="C16" s="13" t="n"/>
+      <c r="D16" s="13" t="n"/>
     </row>
     <row r="17" ht="33" customHeight="1">
       <c r="A17" s="15" t="n">
         <v>14</v>
       </c>
       <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="16" t="n"/>
     </row>
     <row r="18" ht="33" customHeight="1">
       <c r="A18" s="12" t="n">
         <v>15</v>
       </c>
       <c r="B18" s="13" t="n"/>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
     </row>
     <row r="19" ht="33" customHeight="1">
       <c r="A19" s="6" t="n"/>
@@ -1382,6 +1430,8 @@
           <t>CANTEEN WASTE LOG</t>
         </is>
       </c>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="26" t="n"/>
     </row>
     <row r="20" ht="59.25" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
@@ -1391,6 +1441,16 @@
       </c>
       <c r="B20" s="10" t="inlineStr">
         <is>
+          <t>MEALS WASTE (KG)</t>
+        </is>
+      </c>
+      <c r="C20" s="10" t="inlineStr">
+        <is>
+          <t>VEGETABLE WASTE (KG)</t>
+        </is>
+      </c>
+      <c r="D20" s="10" t="inlineStr">
+        <is>
           <t>CARETAKER SIGN</t>
         </is>
       </c>
@@ -1400,90 +1460,120 @@
         <v>16</v>
       </c>
       <c r="B21" s="13" t="n"/>
+      <c r="C21" s="13" t="n"/>
+      <c r="D21" s="13" t="n"/>
     </row>
     <row r="22" ht="33" customHeight="1">
       <c r="A22" s="12" t="n">
         <v>17</v>
       </c>
       <c r="B22" s="13" t="n"/>
+      <c r="C22" s="13" t="n"/>
+      <c r="D22" s="13" t="n"/>
     </row>
     <row r="23" ht="33" customHeight="1">
       <c r="A23" s="12" t="n">
         <v>18</v>
       </c>
       <c r="B23" s="13" t="n"/>
+      <c r="C23" s="13" t="n"/>
+      <c r="D23" s="13" t="n"/>
     </row>
     <row r="24" ht="33" customHeight="1">
       <c r="A24" s="12" t="n">
         <v>19</v>
       </c>
       <c r="B24" s="13" t="n"/>
+      <c r="C24" s="13" t="n"/>
+      <c r="D24" s="13" t="n"/>
     </row>
     <row r="25" ht="33" customHeight="1">
       <c r="A25" s="12" t="n">
         <v>20</v>
       </c>
       <c r="B25" s="13" t="n"/>
+      <c r="C25" s="13" t="n"/>
+      <c r="D25" s="13" t="n"/>
     </row>
     <row r="26" ht="33" customHeight="1">
       <c r="A26" s="15" t="n">
         <v>21</v>
       </c>
       <c r="B26" s="16" t="n"/>
+      <c r="C26" s="16" t="n"/>
+      <c r="D26" s="16" t="n"/>
     </row>
     <row r="27" ht="33" customHeight="1">
       <c r="A27" s="12" t="n">
         <v>22</v>
       </c>
       <c r="B27" s="13" t="n"/>
+      <c r="C27" s="13" t="n"/>
+      <c r="D27" s="13" t="n"/>
     </row>
     <row r="28" ht="33" customHeight="1">
       <c r="A28" s="12" t="n">
         <v>23</v>
       </c>
       <c r="B28" s="13" t="n"/>
+      <c r="C28" s="13" t="n"/>
+      <c r="D28" s="13" t="n"/>
     </row>
     <row r="29" ht="33" customHeight="1">
       <c r="A29" s="12" t="n">
         <v>24</v>
       </c>
       <c r="B29" s="13" t="n"/>
+      <c r="C29" s="13" t="n"/>
+      <c r="D29" s="13" t="n"/>
     </row>
     <row r="30" ht="33" customHeight="1">
       <c r="A30" s="12" t="n">
         <v>25</v>
       </c>
       <c r="B30" s="13" t="n"/>
+      <c r="C30" s="13" t="n"/>
+      <c r="D30" s="13" t="n"/>
     </row>
     <row r="31" ht="33" customHeight="1">
       <c r="A31" s="12" t="n">
         <v>26</v>
       </c>
       <c r="B31" s="13" t="n"/>
+      <c r="C31" s="13" t="n"/>
+      <c r="D31" s="13" t="n"/>
     </row>
     <row r="32" ht="33" customHeight="1">
       <c r="A32" s="12" t="n">
         <v>27</v>
       </c>
       <c r="B32" s="13" t="n"/>
+      <c r="C32" s="13" t="n"/>
+      <c r="D32" s="13" t="n"/>
     </row>
     <row r="33" ht="33" customHeight="1">
       <c r="A33" s="15" t="n">
         <v>28</v>
       </c>
       <c r="B33" s="16" t="n"/>
+      <c r="C33" s="16" t="n"/>
+      <c r="D33" s="16" t="n"/>
     </row>
     <row r="34" ht="33" customHeight="1">
       <c r="A34" s="12" t="n">
         <v>29</v>
       </c>
       <c r="B34" s="13" t="n"/>
+      <c r="C34" s="13" t="n"/>
+      <c r="D34" s="13" t="n"/>
     </row>
     <row r="35" ht="33" customHeight="1" thickBot="1">
       <c r="A35" s="12" t="n">
         <v>30</v>
       </c>
       <c r="B35" s="13" t="n"/>
+      <c r="C35" s="13" t="n"/>
+      <c r="D35" s="13" t="n"/>
     </row>
     <row r="36" ht="33" customHeight="1"/>
     <row r="37" ht="48.75" customHeight="1"/>
@@ -1501,10 +1591,10 @@
     <row r="55" ht="45" customHeight="1"/>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="B1"/>
-    <mergeCell ref="B2"/>
-    <mergeCell ref="B19"/>
-    <mergeCell ref="A1"/>
+    <mergeCell ref="B19:D19"/>
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="D1"/>
+    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>